<commit_message>
Update listedness: NINTEDANIB / Drug intolerance
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1931"/>
+  <dimension ref="A1:D1932"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -35458,6 +35458,24 @@
       </c>
       <c r="D1931" t="inlineStr"/>
     </row>
+    <row r="1932">
+      <c r="A1932" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B1932" t="inlineStr">
+        <is>
+          <t>Drug intolerance</t>
+        </is>
+      </c>
+      <c r="C1932" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1932" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Batch update listedness: 61 added, 1 updated
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1932"/>
+  <dimension ref="A1:D1993"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26196,7 +26196,7 @@
       </c>
       <c r="B1419" t="inlineStr">
         <is>
-          <t xml:space="preserve">Immune-mediated nephritis </t>
+          <t>Immune-mediated nephritis</t>
         </is>
       </c>
       <c r="C1419" t="inlineStr">
@@ -35475,6 +35475,1116 @@
         </is>
       </c>
       <c r="D1932" t="inlineStr"/>
+    </row>
+    <row r="1933">
+      <c r="A1933" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B1933" t="inlineStr">
+        <is>
+          <t>Renal impairment</t>
+        </is>
+      </c>
+      <c r="C1933" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1933" t="inlineStr"/>
+    </row>
+    <row r="1934">
+      <c r="A1934" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B1934" t="inlineStr">
+        <is>
+          <t>Cough</t>
+        </is>
+      </c>
+      <c r="C1934" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1934" t="inlineStr"/>
+    </row>
+    <row r="1935">
+      <c r="A1935" t="inlineStr">
+        <is>
+          <t>RANOLAZINE</t>
+        </is>
+      </c>
+      <c r="B1935" t="inlineStr">
+        <is>
+          <t>Appetite disorder</t>
+        </is>
+      </c>
+      <c r="C1935" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="D1935" t="inlineStr">
+        <is>
+          <t>Check for increased or decreased</t>
+        </is>
+      </c>
+    </row>
+    <row r="1936">
+      <c r="A1936" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B1936" t="inlineStr">
+        <is>
+          <t>Disorientation</t>
+        </is>
+      </c>
+      <c r="C1936" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1936" t="inlineStr"/>
+    </row>
+    <row r="1937">
+      <c r="A1937" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B1937" t="inlineStr">
+        <is>
+          <t>Abdominal distension</t>
+        </is>
+      </c>
+      <c r="C1937" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1937" t="inlineStr"/>
+    </row>
+    <row r="1938">
+      <c r="A1938" t="inlineStr">
+        <is>
+          <t>APIXABAN</t>
+        </is>
+      </c>
+      <c r="B1938" t="inlineStr">
+        <is>
+          <t>Skin atrophy</t>
+        </is>
+      </c>
+      <c r="C1938" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1938" t="inlineStr"/>
+    </row>
+    <row r="1939">
+      <c r="A1939" t="inlineStr">
+        <is>
+          <t>APIXABAN</t>
+        </is>
+      </c>
+      <c r="B1939" t="inlineStr">
+        <is>
+          <t>Increased tendency to bruise</t>
+        </is>
+      </c>
+      <c r="C1939" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1939" t="inlineStr"/>
+    </row>
+    <row r="1940">
+      <c r="A1940" t="inlineStr">
+        <is>
+          <t>PIRFENIDONE</t>
+        </is>
+      </c>
+      <c r="B1940" t="inlineStr">
+        <is>
+          <t>Sensitive skin</t>
+        </is>
+      </c>
+      <c r="C1940" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1940" t="inlineStr"/>
+    </row>
+    <row r="1941">
+      <c r="A1941" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B1941" t="inlineStr">
+        <is>
+          <t>Dyspnoea</t>
+        </is>
+      </c>
+      <c r="C1941" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1941" t="inlineStr"/>
+    </row>
+    <row r="1942">
+      <c r="A1942" t="inlineStr">
+        <is>
+          <t>RIVAROXABAN</t>
+        </is>
+      </c>
+      <c r="B1942" t="inlineStr">
+        <is>
+          <t>Liver function test abnormal</t>
+        </is>
+      </c>
+      <c r="C1942" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="D1942" t="inlineStr"/>
+    </row>
+    <row r="1943">
+      <c r="A1943" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B1943" t="inlineStr">
+        <is>
+          <t>Scrotal inflammation</t>
+        </is>
+      </c>
+      <c r="C1943" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1943" t="inlineStr"/>
+    </row>
+    <row r="1944">
+      <c r="A1944" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B1944" t="inlineStr">
+        <is>
+          <t>Tachycardia</t>
+        </is>
+      </c>
+      <c r="C1944" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1944" t="inlineStr"/>
+    </row>
+    <row r="1945">
+      <c r="A1945" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B1945" t="inlineStr">
+        <is>
+          <t>Tachypnoea</t>
+        </is>
+      </c>
+      <c r="C1945" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1945" t="inlineStr"/>
+    </row>
+    <row r="1946">
+      <c r="A1946" t="inlineStr">
+        <is>
+          <t>PIRFENIDONE</t>
+        </is>
+      </c>
+      <c r="B1946" t="inlineStr">
+        <is>
+          <t>Intentional dose omission</t>
+        </is>
+      </c>
+      <c r="C1946" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1946" t="inlineStr"/>
+    </row>
+    <row r="1947">
+      <c r="A1947" t="inlineStr">
+        <is>
+          <t>ABIRATERONE</t>
+        </is>
+      </c>
+      <c r="B1947" t="inlineStr">
+        <is>
+          <t>Constipation</t>
+        </is>
+      </c>
+      <c r="C1947" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1947" t="inlineStr"/>
+    </row>
+    <row r="1948">
+      <c r="A1948" t="inlineStr">
+        <is>
+          <t>ABIRATERONE</t>
+        </is>
+      </c>
+      <c r="B1948" t="inlineStr">
+        <is>
+          <t>Epistaxis</t>
+        </is>
+      </c>
+      <c r="C1948" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1948" t="inlineStr"/>
+    </row>
+    <row r="1949">
+      <c r="A1949" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B1949" t="inlineStr">
+        <is>
+          <t>Constipation</t>
+        </is>
+      </c>
+      <c r="C1949" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1949" t="inlineStr"/>
+    </row>
+    <row r="1950">
+      <c r="A1950" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B1950" t="inlineStr">
+        <is>
+          <t>Dissociation</t>
+        </is>
+      </c>
+      <c r="C1950" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1950" t="inlineStr"/>
+    </row>
+    <row r="1951">
+      <c r="A1951" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B1951" t="inlineStr">
+        <is>
+          <t>Fall</t>
+        </is>
+      </c>
+      <c r="C1951" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1951" t="inlineStr"/>
+    </row>
+    <row r="1952">
+      <c r="A1952" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B1952" t="inlineStr">
+        <is>
+          <t>Scrotal swelling</t>
+        </is>
+      </c>
+      <c r="C1952" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1952" t="inlineStr"/>
+    </row>
+    <row r="1953">
+      <c r="A1953" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B1953" t="inlineStr">
+        <is>
+          <t>Lichen sclerosus</t>
+        </is>
+      </c>
+      <c r="C1953" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1953" t="inlineStr"/>
+    </row>
+    <row r="1954">
+      <c r="A1954" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B1954" t="inlineStr">
+        <is>
+          <t>Chills</t>
+        </is>
+      </c>
+      <c r="C1954" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1954" t="inlineStr"/>
+    </row>
+    <row r="1955">
+      <c r="A1955" t="inlineStr">
+        <is>
+          <t>SITAGLIPTIN</t>
+        </is>
+      </c>
+      <c r="B1955" t="inlineStr">
+        <is>
+          <t>Muscle spasms</t>
+        </is>
+      </c>
+      <c r="C1955" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1955" t="inlineStr"/>
+    </row>
+    <row r="1956">
+      <c r="A1956" t="inlineStr">
+        <is>
+          <t>APREMILAST</t>
+        </is>
+      </c>
+      <c r="B1956" t="inlineStr">
+        <is>
+          <t>Drug ineffective</t>
+        </is>
+      </c>
+      <c r="C1956" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1956" t="inlineStr"/>
+    </row>
+    <row r="1957">
+      <c r="A1957" t="inlineStr">
+        <is>
+          <t>SAFINAMIDE</t>
+        </is>
+      </c>
+      <c r="B1957" t="inlineStr">
+        <is>
+          <t>Diarrhoea</t>
+        </is>
+      </c>
+      <c r="C1957" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="D1957" t="inlineStr"/>
+    </row>
+    <row r="1958">
+      <c r="A1958" t="inlineStr">
+        <is>
+          <t>SAFINAMIDE</t>
+        </is>
+      </c>
+      <c r="B1958" t="inlineStr">
+        <is>
+          <t>Dizziness</t>
+        </is>
+      </c>
+      <c r="C1958" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="D1958" t="inlineStr"/>
+    </row>
+    <row r="1959">
+      <c r="A1959" t="inlineStr">
+        <is>
+          <t>RIVAROXABAN</t>
+        </is>
+      </c>
+      <c r="B1959" t="inlineStr">
+        <is>
+          <t>Iron deficiency anaemia</t>
+        </is>
+      </c>
+      <c r="C1959" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="D1959" t="inlineStr"/>
+    </row>
+    <row r="1960">
+      <c r="A1960" t="inlineStr">
+        <is>
+          <t>ABIRATERONE</t>
+        </is>
+      </c>
+      <c r="B1960" t="inlineStr">
+        <is>
+          <t>Dry skin</t>
+        </is>
+      </c>
+      <c r="C1960" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1960" t="inlineStr"/>
+    </row>
+    <row r="1961">
+      <c r="A1961" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B1961" t="inlineStr">
+        <is>
+          <t>Photopsia</t>
+        </is>
+      </c>
+      <c r="C1961" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1961" t="inlineStr"/>
+    </row>
+    <row r="1962">
+      <c r="A1962" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B1962" t="inlineStr">
+        <is>
+          <t>Glucose urine</t>
+        </is>
+      </c>
+      <c r="C1962" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1962" t="inlineStr"/>
+    </row>
+    <row r="1963">
+      <c r="A1963" t="inlineStr">
+        <is>
+          <t>ABIRATERONE</t>
+        </is>
+      </c>
+      <c r="B1963" t="inlineStr">
+        <is>
+          <t>Nausea</t>
+        </is>
+      </c>
+      <c r="C1963" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1963" t="inlineStr"/>
+    </row>
+    <row r="1964">
+      <c r="A1964" t="inlineStr">
+        <is>
+          <t>PIRFENIDONE</t>
+        </is>
+      </c>
+      <c r="B1964" t="inlineStr">
+        <is>
+          <t>Quality of life decreased</t>
+        </is>
+      </c>
+      <c r="C1964" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1964" t="inlineStr"/>
+    </row>
+    <row r="1965">
+      <c r="A1965" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B1965" t="inlineStr">
+        <is>
+          <t>Vulvovaginal erythema</t>
+        </is>
+      </c>
+      <c r="C1965" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1965" t="inlineStr"/>
+    </row>
+    <row r="1966">
+      <c r="A1966" t="inlineStr">
+        <is>
+          <t>FAMOTIDINE</t>
+        </is>
+      </c>
+      <c r="B1966" t="inlineStr">
+        <is>
+          <t>Asthenia</t>
+        </is>
+      </c>
+      <c r="C1966" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1966" t="inlineStr"/>
+    </row>
+    <row r="1967">
+      <c r="A1967" t="inlineStr">
+        <is>
+          <t>PIRFENIDONE</t>
+        </is>
+      </c>
+      <c r="B1967" t="inlineStr">
+        <is>
+          <t>Haemochromatosis</t>
+        </is>
+      </c>
+      <c r="C1967" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1967" t="inlineStr"/>
+    </row>
+    <row r="1968">
+      <c r="A1968" t="inlineStr">
+        <is>
+          <t>ABIRATERONE</t>
+        </is>
+      </c>
+      <c r="B1968" t="inlineStr">
+        <is>
+          <t>Urinary incontinence</t>
+        </is>
+      </c>
+      <c r="C1968" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1968" t="inlineStr"/>
+    </row>
+    <row r="1969">
+      <c r="A1969" t="inlineStr">
+        <is>
+          <t>APREMILAST</t>
+        </is>
+      </c>
+      <c r="B1969" t="inlineStr">
+        <is>
+          <t>Arthralgia</t>
+        </is>
+      </c>
+      <c r="C1969" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1969" t="inlineStr"/>
+    </row>
+    <row r="1970">
+      <c r="A1970" t="inlineStr">
+        <is>
+          <t>APREMILAST</t>
+        </is>
+      </c>
+      <c r="B1970" t="inlineStr">
+        <is>
+          <t>Dysgeusia</t>
+        </is>
+      </c>
+      <c r="C1970" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1970" t="inlineStr"/>
+    </row>
+    <row r="1971">
+      <c r="A1971" t="inlineStr">
+        <is>
+          <t>FAMOTIDINE</t>
+        </is>
+      </c>
+      <c r="B1971" t="inlineStr">
+        <is>
+          <t>Mania</t>
+        </is>
+      </c>
+      <c r="C1971" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1971" t="inlineStr"/>
+    </row>
+    <row r="1972">
+      <c r="A1972" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B1972" t="inlineStr">
+        <is>
+          <t>Feeling abnormal</t>
+        </is>
+      </c>
+      <c r="C1972" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1972" t="inlineStr"/>
+    </row>
+    <row r="1973">
+      <c r="A1973" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B1973" t="inlineStr">
+        <is>
+          <t>Haemorrhage intracranial</t>
+        </is>
+      </c>
+      <c r="C1973" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1973" t="inlineStr"/>
+    </row>
+    <row r="1974">
+      <c r="A1974" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B1974" t="inlineStr">
+        <is>
+          <t>Ulcer</t>
+        </is>
+      </c>
+      <c r="C1974" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1974" t="inlineStr"/>
+    </row>
+    <row r="1975">
+      <c r="A1975" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B1975" t="inlineStr">
+        <is>
+          <t>Coma scale abnormal</t>
+        </is>
+      </c>
+      <c r="C1975" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1975" t="inlineStr"/>
+    </row>
+    <row r="1976">
+      <c r="A1976" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B1976" t="inlineStr">
+        <is>
+          <t>Oedema peripheral</t>
+        </is>
+      </c>
+      <c r="C1976" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1976" t="inlineStr"/>
+    </row>
+    <row r="1977">
+      <c r="A1977" t="inlineStr">
+        <is>
+          <t>ABIRATERONE</t>
+        </is>
+      </c>
+      <c r="B1977" t="inlineStr">
+        <is>
+          <t>Dysphagia</t>
+        </is>
+      </c>
+      <c r="C1977" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1977" t="inlineStr"/>
+    </row>
+    <row r="1978">
+      <c r="A1978" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B1978" t="inlineStr">
+        <is>
+          <t>Thermal burns of eye</t>
+        </is>
+      </c>
+      <c r="C1978" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1978" t="inlineStr"/>
+    </row>
+    <row r="1979">
+      <c r="A1979" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B1979" t="inlineStr">
+        <is>
+          <t>Eye pruritus</t>
+        </is>
+      </c>
+      <c r="C1979" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1979" t="inlineStr"/>
+    </row>
+    <row r="1980">
+      <c r="A1980" t="inlineStr">
+        <is>
+          <t>APIXABAN</t>
+        </is>
+      </c>
+      <c r="B1980" t="inlineStr">
+        <is>
+          <t>Drug intolerance</t>
+        </is>
+      </c>
+      <c r="C1980" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1980" t="inlineStr">
+        <is>
+          <t>Check for specific type of intolerance</t>
+        </is>
+      </c>
+    </row>
+    <row r="1981">
+      <c r="A1981" t="inlineStr">
+        <is>
+          <t>APIXABAN</t>
+        </is>
+      </c>
+      <c r="B1981" t="inlineStr">
+        <is>
+          <t>Swelling</t>
+        </is>
+      </c>
+      <c r="C1981" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1981" t="inlineStr"/>
+    </row>
+    <row r="1982">
+      <c r="A1982" t="inlineStr">
+        <is>
+          <t>PIRFENIDONE</t>
+        </is>
+      </c>
+      <c r="B1982" t="inlineStr">
+        <is>
+          <t>Surgery</t>
+        </is>
+      </c>
+      <c r="C1982" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1982" t="inlineStr"/>
+    </row>
+    <row r="1983">
+      <c r="A1983" t="inlineStr">
+        <is>
+          <t>APIXABAN</t>
+        </is>
+      </c>
+      <c r="B1983" t="inlineStr">
+        <is>
+          <t>Dermatitis bullous</t>
+        </is>
+      </c>
+      <c r="C1983" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1983" t="inlineStr"/>
+    </row>
+    <row r="1984">
+      <c r="A1984" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B1984" t="inlineStr">
+        <is>
+          <t>Liver function test</t>
+        </is>
+      </c>
+      <c r="C1984" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="D1984" t="inlineStr"/>
+    </row>
+    <row r="1985">
+      <c r="A1985" t="inlineStr">
+        <is>
+          <t>PIRFENIDONE</t>
+        </is>
+      </c>
+      <c r="B1985" t="inlineStr">
+        <is>
+          <t>Disease progression</t>
+        </is>
+      </c>
+      <c r="C1985" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1985" t="inlineStr"/>
+    </row>
+    <row r="1986">
+      <c r="A1986" t="inlineStr">
+        <is>
+          <t>PIRFENIDONE</t>
+        </is>
+      </c>
+      <c r="B1986" t="inlineStr">
+        <is>
+          <t>Speech disorder</t>
+        </is>
+      </c>
+      <c r="C1986" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1986" t="inlineStr"/>
+    </row>
+    <row r="1987">
+      <c r="A1987" t="inlineStr">
+        <is>
+          <t>APIXABAN</t>
+        </is>
+      </c>
+      <c r="B1987" t="inlineStr">
+        <is>
+          <t>Haematoma muscle</t>
+        </is>
+      </c>
+      <c r="C1987" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="D1987" t="inlineStr"/>
+    </row>
+    <row r="1988">
+      <c r="A1988" t="inlineStr">
+        <is>
+          <t>PIRFENIDONE</t>
+        </is>
+      </c>
+      <c r="B1988" t="inlineStr">
+        <is>
+          <t>Visual impairment</t>
+        </is>
+      </c>
+      <c r="C1988" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1988" t="inlineStr"/>
+    </row>
+    <row r="1989">
+      <c r="A1989" t="inlineStr">
+        <is>
+          <t>PIRFENIDONE</t>
+        </is>
+      </c>
+      <c r="B1989" t="inlineStr">
+        <is>
+          <t>Stomatitis</t>
+        </is>
+      </c>
+      <c r="C1989" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1989" t="inlineStr"/>
+    </row>
+    <row r="1990">
+      <c r="A1990" t="inlineStr">
+        <is>
+          <t>RIVAROXABAN</t>
+        </is>
+      </c>
+      <c r="B1990" t="inlineStr">
+        <is>
+          <t>Swollen tongue</t>
+        </is>
+      </c>
+      <c r="C1990" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1990" t="inlineStr">
+        <is>
+          <t>Listed along with Angiodema</t>
+        </is>
+      </c>
+    </row>
+    <row r="1991">
+      <c r="A1991" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B1991" t="inlineStr">
+        <is>
+          <t>Paraesthesia oral</t>
+        </is>
+      </c>
+      <c r="C1991" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1991" t="inlineStr"/>
+    </row>
+    <row r="1992">
+      <c r="A1992" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B1992" t="inlineStr">
+        <is>
+          <t>Pulmonary fibrosis</t>
+        </is>
+      </c>
+      <c r="C1992" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1992" t="inlineStr"/>
+    </row>
+    <row r="1993">
+      <c r="A1993" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B1993" t="inlineStr">
+        <is>
+          <t>Rheumatoid arthritis</t>
+        </is>
+      </c>
+      <c r="C1993" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1993" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Batch update listedness: 0 added, 4 updated
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -12078,7 +12078,11 @@
           <t>Unexpected</t>
         </is>
       </c>
-      <c r="D638" t="inlineStr"/>
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="639">
       <c r="A639" t="inlineStr">
@@ -35640,7 +35644,11 @@
           <t>Unexpected</t>
         </is>
       </c>
-      <c r="D1941" t="inlineStr"/>
+      <c r="D1941" t="inlineStr">
+        <is>
+          <t>Listed only with DKA</t>
+        </is>
+      </c>
     </row>
     <row r="1942">
       <c r="A1942" t="inlineStr">
@@ -35676,7 +35684,11 @@
           <t>Unexpected</t>
         </is>
       </c>
-      <c r="D1943" t="inlineStr"/>
+      <c r="D1943" t="inlineStr">
+        <is>
+          <t>Listed with Fournier's gangrene</t>
+        </is>
+      </c>
     </row>
     <row r="1944">
       <c r="A1944" t="inlineStr">

</xml_diff>

<commit_message>
Batch update listedness: 0 added, 3 updated
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -12075,14 +12075,10 @@
       </c>
       <c r="C638" t="inlineStr">
         <is>
-          <t>Unexpected</t>
-        </is>
-      </c>
-      <c r="D638" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="D638" t="inlineStr"/>
     </row>
     <row r="639">
       <c r="A639" t="inlineStr">
@@ -26312,12 +26308,12 @@
       </c>
       <c r="B1425" t="inlineStr">
         <is>
-          <t xml:space="preserve">Joint swelling </t>
+          <t>Joint swelling</t>
         </is>
       </c>
       <c r="C1425" t="inlineStr">
         <is>
-          <t>Unxpected</t>
+          <t>Unexpected</t>
         </is>
       </c>
       <c r="D1425" t="inlineStr">

</xml_diff>

<commit_message>
Update listedness: ABIRATERONE / Odynophagia
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1993"/>
+  <dimension ref="A1:D1994"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36594,6 +36594,24 @@
       </c>
       <c r="D1993" t="inlineStr"/>
     </row>
+    <row r="1994">
+      <c r="A1994" t="inlineStr">
+        <is>
+          <t>ABIRATERONE</t>
+        </is>
+      </c>
+      <c r="B1994" t="inlineStr">
+        <is>
+          <t>Odynophagia</t>
+        </is>
+      </c>
+      <c r="C1994" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1994" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: PIRFENIDONE / Psychogenic loss of appetite
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1994"/>
+  <dimension ref="A1:D1995"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36612,6 +36612,24 @@
       </c>
       <c r="D1994" t="inlineStr"/>
     </row>
+    <row r="1995">
+      <c r="A1995" t="inlineStr">
+        <is>
+          <t>PIRFENIDONE</t>
+        </is>
+      </c>
+      <c r="B1995" t="inlineStr">
+        <is>
+          <t>Psychogenic loss of appetite</t>
+        </is>
+      </c>
+      <c r="C1995" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="D1995" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: PIRFENIDONE / Oropharyngeal pain
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1995"/>
+  <dimension ref="A1:D1996"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36630,6 +36630,24 @@
       </c>
       <c r="D1995" t="inlineStr"/>
     </row>
+    <row r="1996">
+      <c r="A1996" t="inlineStr">
+        <is>
+          <t>PIRFENIDONE</t>
+        </is>
+      </c>
+      <c r="B1996" t="inlineStr">
+        <is>
+          <t>Oropharyngeal pain</t>
+        </is>
+      </c>
+      <c r="C1996" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1996" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: PIRFENIDONE / Dry throat
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1996"/>
+  <dimension ref="A1:D1997"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36648,6 +36648,24 @@
       </c>
       <c r="D1996" t="inlineStr"/>
     </row>
+    <row r="1997">
+      <c r="A1997" t="inlineStr">
+        <is>
+          <t>PIRFENIDONE</t>
+        </is>
+      </c>
+      <c r="B1997" t="inlineStr">
+        <is>
+          <t>Dry throat</t>
+        </is>
+      </c>
+      <c r="C1997" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1997" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: RIVAROXABAN / Depressed mood
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1997"/>
+  <dimension ref="A1:D1998"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36666,6 +36666,24 @@
       </c>
       <c r="D1997" t="inlineStr"/>
     </row>
+    <row r="1998">
+      <c r="A1998" t="inlineStr">
+        <is>
+          <t>RIVAROXABAN</t>
+        </is>
+      </c>
+      <c r="B1998" t="inlineStr">
+        <is>
+          <t>Depressed mood</t>
+        </is>
+      </c>
+      <c r="C1998" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D1998" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: RIVAROXABAN / Tension headache
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1998"/>
+  <dimension ref="A1:D1999"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36684,6 +36684,24 @@
       </c>
       <c r="D1998" t="inlineStr"/>
     </row>
+    <row r="1999">
+      <c r="A1999" t="inlineStr">
+        <is>
+          <t>RIVAROXABAN</t>
+        </is>
+      </c>
+      <c r="B1999" t="inlineStr">
+        <is>
+          <t>Tension headache</t>
+        </is>
+      </c>
+      <c r="C1999" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="D1999" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: RIVAROXABAN / Tachyphrenia
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1999"/>
+  <dimension ref="A1:D2000"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36702,6 +36702,24 @@
       </c>
       <c r="D1999" t="inlineStr"/>
     </row>
+    <row r="2000">
+      <c r="A2000" t="inlineStr">
+        <is>
+          <t>RIVAROXABAN</t>
+        </is>
+      </c>
+      <c r="B2000" t="inlineStr">
+        <is>
+          <t>Tachyphrenia</t>
+        </is>
+      </c>
+      <c r="C2000" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2000" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: NINTEDANIB / Apathy
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2000"/>
+  <dimension ref="A1:D2001"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36720,6 +36720,24 @@
       </c>
       <c r="D2000" t="inlineStr"/>
     </row>
+    <row r="2001">
+      <c r="A2001" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B2001" t="inlineStr">
+        <is>
+          <t>Apathy</t>
+        </is>
+      </c>
+      <c r="C2001" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2001" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: FAMOTIDINE / Skin irritation
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2001"/>
+  <dimension ref="A1:D2002"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36738,6 +36738,24 @@
       </c>
       <c r="D2001" t="inlineStr"/>
     </row>
+    <row r="2002">
+      <c r="A2002" t="inlineStr">
+        <is>
+          <t>FAMOTIDINE</t>
+        </is>
+      </c>
+      <c r="B2002" t="inlineStr">
+        <is>
+          <t>Skin irritation</t>
+        </is>
+      </c>
+      <c r="C2002" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2002" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: APIXABAN / Dyspepsia
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2002"/>
+  <dimension ref="A1:D2003"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36756,6 +36756,24 @@
       </c>
       <c r="D2002" t="inlineStr"/>
     </row>
+    <row r="2003">
+      <c r="A2003" t="inlineStr">
+        <is>
+          <t>APIXABAN</t>
+        </is>
+      </c>
+      <c r="B2003" t="inlineStr">
+        <is>
+          <t>Dyspepsia</t>
+        </is>
+      </c>
+      <c r="C2003" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2003" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>